<commit_message>
edited excel sheet with new SIQs
</commit_message>
<xml_diff>
--- a/SIQs.xlsx
+++ b/SIQs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ITI\iti-Config-managment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1BA9AF7-32BB-4D22-AD15-1797A2B25E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950546A1-4C03-4886-96E5-5656F6BB7E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B6544A6E-4D41-4CEF-9174-6A1D4B9FF080}"/>
   </bookViews>
@@ -37,19 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
-  <si>
-    <t>Column5</t>
-  </si>
-  <si>
-    <t>Column6</t>
-  </si>
-  <si>
-    <t>Column7</t>
-  </si>
-  <si>
-    <t>Column8</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
   <si>
     <t>ID</t>
   </si>
@@ -108,21 +96,6 @@
     <t>Req_SIQ_16</t>
   </si>
   <si>
-    <t>Req_SIQ_17</t>
-  </si>
-  <si>
-    <t>Req_SIQ_18</t>
-  </si>
-  <si>
-    <t>Req_SIQ_19</t>
-  </si>
-  <si>
-    <t>Req_SIQ_20</t>
-  </si>
-  <si>
-    <t>Req_SIQ_21</t>
-  </si>
-  <si>
     <t>the client can only buy or buy and sell?</t>
   </si>
   <si>
@@ -135,9 +108,6 @@
     <t>supplier should appear in the purchasing process or just to the admin</t>
   </si>
   <si>
-    <t>payment goes to the store directly either with cash or visa</t>
-  </si>
-  <si>
     <t>Proposed answer</t>
   </si>
   <si>
@@ -156,31 +126,10 @@
     <t>yes</t>
   </si>
   <si>
-    <t>Secure Login  means using email and password</t>
-  </si>
-  <si>
-    <t>registeration form</t>
-  </si>
-  <si>
     <t>should have first name, last name, email and password</t>
   </si>
   <si>
     <t>web page language is english</t>
-  </si>
-  <si>
-    <t>Req_SIQ_</t>
-  </si>
-  <si>
-    <t>validate password</t>
-  </si>
-  <si>
-    <t>validate first name</t>
-  </si>
-  <si>
-    <t>validate last name</t>
-  </si>
-  <si>
-    <t>validate registeration email</t>
   </si>
   <si>
     <t>not empty
@@ -195,15 +144,9 @@
 must be not be blank</t>
   </si>
   <si>
-    <t xml:space="preserve">invalid data in registeration </t>
-  </si>
-  <si>
     <t>pop up showing "invalid data"</t>
   </si>
   <si>
-    <t xml:space="preserve">invalid mail or password in log in </t>
-  </si>
-  <si>
     <t>pop up showing "invalid mail or password"</t>
   </si>
   <si>
@@ -214,6 +157,40 @@
   </si>
   <si>
     <t>bngrab git hub</t>
+  </si>
+  <si>
+    <t>Req_SIQ_6</t>
+  </si>
+  <si>
+    <t>what are the nesseccary data for registeration?</t>
+  </si>
+  <si>
+    <t>what does secure log in means?</t>
+  </si>
+  <si>
+    <t>Login using email and password</t>
+  </si>
+  <si>
+    <t>how to confirm password?</t>
+  </si>
+  <si>
+    <t>how to confirm that first name is correct?</t>
+  </si>
+  <si>
+    <t>how to confirm that last name is correct?</t>
+  </si>
+  <si>
+    <t>how to confirm on registeration email?</t>
+  </si>
+  <si>
+    <t>what happens when entering wrong data in registeration?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">what happens when entering wrong mail or password in log in? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">what should be the first page to appear upon accessing the website?
+</t>
   </si>
 </sst>
 </file>
@@ -284,75 +261,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <font>
         <b val="0"/>
@@ -472,18 +381,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{21609EFC-225A-40B5-91D1-9A1DC34E4AA8}" name="Table1" displayName="Table1" ref="A1:I44" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I44" xr:uid="{21609EFC-225A-40B5-91D1-9A1DC34E4AA8}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{6AC48E7B-7415-46DB-9EBC-FE642573AA3D}" name="ID" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{FD9CA64D-4124-4A9B-8E27-B1B73ADB1CAA}" name="Question" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{18372005-390C-4765-BDB9-A49F33E6B4D4}" name="Proposed answer" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{2E9C5D18-DD1B-47ED-A7F9-1BFE8FC18C96}" name=" Customer answer" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{A0D1BD0B-7D24-44FB-A66A-0E3329BC2DC4}" name="Status" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{7069F9BD-C555-4D63-B183-39EDC5C19641}" name="Column5" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{0B8AA333-784D-4166-8969-CC57645DA53C}" name="Column6" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{0C856E16-9ED8-44FB-A0C3-18DD7261CCA9}" name="Column7" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{EE79C7D6-8CB2-4047-A3EC-242865EFB643}" name="Column8" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{21609EFC-225A-40B5-91D1-9A1DC34E4AA8}" name="Table1" displayName="Table1" ref="A1:E44" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E44" xr:uid="{21609EFC-225A-40B5-91D1-9A1DC34E4AA8}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{6AC48E7B-7415-46DB-9EBC-FE642573AA3D}" name="ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{FD9CA64D-4124-4A9B-8E27-B1B73ADB1CAA}" name="Question" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{18372005-390C-4765-BDB9-A49F33E6B4D4}" name="Proposed answer" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2E9C5D18-DD1B-47ED-A7F9-1BFE8FC18C96}" name=" Customer answer" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{A0D1BD0B-7D24-44FB-A66A-0E3329BC2DC4}" name="Status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -806,621 +711,426 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2F2C9DE-B329-40FD-AE6F-FBEC99EE2B97}">
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.77734375" customWidth="1"/>
     <col min="2" max="2" width="31.44140625" customWidth="1"/>
     <col min="3" max="3" width="26.6640625" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="5" max="9" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:10" ht="60" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
+    </row>
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="B5" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
+    </row>
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" ht="45" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
+    </row>
+    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>39</v>
+      </c>
       <c r="B7" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
+    </row>
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="B8" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
+    </row>
+    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="B9" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:10" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" ht="75" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
+    </row>
+    <row r="14" spans="1:10" ht="60" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="B14" s="1" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
+    </row>
+    <row r="15" spans="1:10" ht="15" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:10" ht="15" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" ht="45" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:5" ht="45" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>15</v>
-      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>16</v>
-      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>17</v>
-      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-    </row>
-    <row r="21" spans="1:9" ht="45" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>18</v>
-      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A21" s="1"/>
       <c r="B21" s="1"/>
-      <c r="C21" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-    </row>
-    <row r="22" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>19</v>
-      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-    </row>
-    <row r="23" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>20</v>
-      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-    </row>
-    <row r="24" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>21</v>
-      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-    </row>
-    <row r="25" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>22</v>
-      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-    </row>
-    <row r="26" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>23</v>
-      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-    </row>
-    <row r="27" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>24</v>
-      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-    </row>
-    <row r="28" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>25</v>
-      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-    </row>
-    <row r="29" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>26</v>
-      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-    </row>
-    <row r="30" spans="1:9" ht="15" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>27</v>
-      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-    </row>
-    <row r="31" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-    </row>
-    <row r="32" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-    </row>
-    <row r="33" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-    </row>
-    <row r="34" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-    </row>
-    <row r="35" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-    </row>
-    <row r="36" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-    </row>
-    <row r="37" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-    </row>
-    <row r="38" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-    </row>
-    <row r="39" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
-      <c r="H39" s="1"/>
-      <c r="I39" s="1"/>
-    </row>
-    <row r="40" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-    </row>
-    <row r="41" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
-      <c r="H41" s="1"/>
-      <c r="I41" s="1"/>
-    </row>
-    <row r="42" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-    </row>
-    <row r="43" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
-      <c r="H43" s="1"/>
-      <c r="I43" s="1"/>
-    </row>
-    <row r="44" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
-      <c r="G44" s="1"/>
-      <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
edited siqs khalena nekhlas
</commit_message>
<xml_diff>
--- a/SIQs.xlsx
+++ b/SIQs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ITI\iti-Config-managment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0D95731-1CF0-474A-8850-1F0AA541DEF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20303508-84BC-4A6B-AF3D-B4D4958ECA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B6544A6E-4D41-4CEF-9174-6A1D4B9FF080}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="68">
   <si>
     <t>ID</t>
   </si>
@@ -178,9 +178,6 @@
 </t>
   </si>
   <si>
-    <t>can admin add or delete client and supplier accounts?</t>
-  </si>
-  <si>
     <t>what does product page contains?</t>
   </si>
   <si>
@@ -200,6 +197,56 @@
   </si>
   <si>
     <t>LOGIN FEATURE</t>
+  </si>
+  <si>
+    <t>CLIENT FEATURES</t>
+  </si>
+  <si>
+    <t>what does home page contain?</t>
+  </si>
+  <si>
+    <t>products and their title and image</t>
+  </si>
+  <si>
+    <t>what are the supplier's features?</t>
+  </si>
+  <si>
+    <t>can add product with the title, description, image and price
+and can delete his products</t>
+  </si>
+  <si>
+    <t>SUPPLIER FEATURES</t>
+  </si>
+  <si>
+    <t>ADMIN FEATURES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">what should be in the dashboard of the admin?
+</t>
+  </si>
+  <si>
+    <t>a list of the existing clients and suppliers</t>
+  </si>
+  <si>
+    <t>can admin add or delete and supplier accounts?</t>
+  </si>
+  <si>
+    <t>can admin delete an existing client account?</t>
+  </si>
+  <si>
+    <t>Req_SIQ_17</t>
+  </si>
+  <si>
+    <t>Req_SIQ_18</t>
+  </si>
+  <si>
+    <t>WEB PAGE FEATURES</t>
+  </si>
+  <si>
+    <t>Req_SIQ_19</t>
+  </si>
+  <si>
+    <t>Req_SIQ_20</t>
   </si>
 </sst>
 </file>
@@ -272,14 +319,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -405,8 +452,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{21609EFC-225A-40B5-91D1-9A1DC34E4AA8}" name="Table1" displayName="Table1" ref="A1:E46" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:E46" xr:uid="{21609EFC-225A-40B5-91D1-9A1DC34E4AA8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{21609EFC-225A-40B5-91D1-9A1DC34E4AA8}" name="Table1" displayName="Table1" ref="A1:E44" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E44" xr:uid="{21609EFC-225A-40B5-91D1-9A1DC34E4AA8}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{6AC48E7B-7415-46DB-9EBC-FE642573AA3D}" name="ID" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{FD9CA64D-4124-4A9B-8E27-B1B73ADB1CAA}" name="Question" dataDxfId="3"/>
@@ -735,7 +782,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2F2C9DE-B329-40FD-AE6F-FBEC99EE2B97}">
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.77734375" customWidth="1"/>
@@ -763,13 +810,13 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
+      <c r="A2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -783,13 +830,13 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
     </row>
     <row r="4" spans="1:12" ht="60" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>38</v>
@@ -802,7 +849,7 @@
     </row>
     <row r="5" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>39</v>
@@ -815,7 +862,7 @@
     </row>
     <row r="6" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>40</v>
@@ -828,7 +875,7 @@
     </row>
     <row r="7" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>41</v>
@@ -841,7 +888,7 @@
     </row>
     <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>42</v>
@@ -852,229 +899,240 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="10" spans="1:12" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+    </row>
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="J10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
+    </row>
+    <row r="11" spans="1:12" ht="45" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:12" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-    </row>
-    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.3">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:12" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+    <row r="14" spans="1:12" ht="45" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:12" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="60" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:12" ht="45" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="30" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="1:5" ht="60" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>33</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="75" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:10" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:5" ht="45" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="B21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="1"/>
+        <v>61</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
+    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-    </row>
-    <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
+    <row r="25" spans="1:10" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+    </row>
+    <row r="26" spans="1:10" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-    </row>
-    <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
+      <c r="J26" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-    </row>
-    <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-    </row>
-    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
-    </row>
-    <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-    </row>
-    <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -1159,20 +1217,6 @@
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
-    </row>
-    <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="1"/>
-      <c r="E45" s="1"/>
-    </row>
-    <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.3">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>